<commit_message>
feat(loans): bootstrap fair rates by segment
Redeem remaining principal at each segment end and lock its solved
coupon/spread before extending to the next boundary.

Expose fair_rates in Rust/Python and spill it from QS.FAIR.RATE,
with optional transpose. Preserve scalar results for single-segment loans.
</commit_message>
<xml_diff>
--- a/bindings/excel/examples/loan_pricing_example.xlsx
+++ b/bindings/excel/examples/loan_pricing_example.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="103">
   <si>
     <t>Loans: monthly payments, prepayment, borrower credit, and funding</t>
   </si>
@@ -65,7 +65,7 @@
     <t>Funding discount factors multiply EURIBOR12m by a separate treasury-spread curve.</t>
   </si>
   <si>
-    <t>FairRate solves a uniform fixed coupon or floating margin at origination. Introductory/bounded schedules omit this unsupported solve.</t>
+    <t>FairRate bootstraps each rate segment: repay remaining capital at its end, solve, lock, and extend. Arrays are transposed into a row; bounded coupons omit the solve.</t>
   </si>
   <si>
     <t>Cashflows include scheduled receipts, prepayments, and recovery in legs 0, 1, and 2. Bounded coupons exclude option time value.</t>
@@ -242,7 +242,13 @@
     <t>PV less advance</t>
   </si>
   <si>
-    <t>Fair coupon / spread</t>
+    <t>Fair first segment</t>
+  </si>
+  <si>
+    <t>Fair second segment</t>
+  </si>
+  <si>
+    <t>Fair third segment</t>
   </si>
   <si>
     <t>French</t>
@@ -278,15 +284,15 @@
     <t>{"introductory_periods": 60, "introductory_rate": 0.04}</t>
   </si>
   <si>
-    <t>Unsupported for mixed/bounded coupons</t>
-  </si>
-  <si>
     <t>Bounded floating</t>
   </si>
   <si>
     <t>{"amortization_rate": 0.05, "floor": 0.02, "cap": 0.045}</t>
   </si>
   <si>
+    <t>Unsupported for bounded coupons</t>
+  </si>
+  <si>
     <t>15% annual CPR</t>
   </si>
   <si>
@@ -309,6 +315,18 @@
   </si>
   <si>
     <t>{"amortization_rate": 0.05, "discount_index": {"Other": "FUNDING"}}</t>
+  </si>
+  <si>
+    <t>Stepped fixed</t>
+  </si>
+  <si>
+    <t>{"coupon_segments": [{"rate": 0.03, "periods": 60}, {"rate": 0.04, "periods": 60}, {"rate": 0.05}]}</t>
+  </si>
+  <si>
+    <t>Stepped then floating</t>
+  </si>
+  <si>
+    <t>{"coupon_segments": [{"rate": 0.03, "periods": 60}, {"rate": 0.04, "periods": 60}, {"rate": 0.01, "market_index": "EURIBOR12m"}]}</t>
   </si>
   <si>
     <t>French contractual receipts</t>
@@ -1195,17 +1213,19 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A4:L14"/>
+  <dimension ref="A4:L16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="31.7109375" customWidth="1"/>
     <col min="2" max="4" width="22.7109375" style="1" customWidth="1"/>
     <col min="5" max="5" width="70.7109375" customWidth="1"/>
     <col min="6" max="6" width="48.7109375" customWidth="1"/>
-    <col min="7" max="12" width="22.7109375" style="1" customWidth="1"/>
+    <col min="7" max="8" width="22.7109375" style="1" customWidth="1"/>
+    <col min="9" max="11" width="21.7109375" style="6" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:11">
       <c r="A4" s="4" t="s">
         <v>58</v>
       </c>
@@ -1233,10 +1253,16 @@
       <c r="I4" s="4" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="5" spans="1:9">
+      <c r="J4" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B5" s="6">
         <f>'Loan Inputs'!B5</f>
@@ -1244,10 +1270,10 @@
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F5" cm="1">
         <f t="array" ref="F5">_xll.QS.TRADE.LOAN("Loans.Case5",Market!$B$3,'Loan Inputs'!$B$7,'Loan Inputs'!$B$8,'Loan Inputs'!$B$11,'Loan Inputs'!$B$4,B5,C5,D5,'Loan Inputs'!$B$9,'Loan Inputs'!$B$10,"Receive",E5)</f>
@@ -1262,13 +1288,13 @@
         <v>0</v>
       </c>
       <c r="I5" s="6" cm="1">
-        <f t="array" ref="I5">_xll.QS.FAIR.RATE(F5,Market!$F$11)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
+        <f t="array" ref="I5">_xll.QS.FAIR.RATE(F5,Market!$F$11,TRUE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B6" s="6">
         <f>'Loan Inputs'!B5</f>
@@ -1276,10 +1302,10 @@
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F6" cm="1">
         <f t="array" ref="F6">_xll.QS.TRADE.LOAN("Loans.Case6",Market!$B$3,'Loan Inputs'!$B$7,'Loan Inputs'!$B$8,'Loan Inputs'!$B$11,'Loan Inputs'!$B$4,B6,C6,D6,'Loan Inputs'!$B$9,'Loan Inputs'!$B$10,"Receive",E6)</f>
@@ -1294,13 +1320,13 @@
         <v>0</v>
       </c>
       <c r="I6" s="6" cm="1">
-        <f t="array" ref="I6">_xll.QS.FAIR.RATE(F6,Market!$F$11)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
+        <f t="array" ref="I6">_xll.QS.FAIR.RATE(F6,Market!$F$11,TRUE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B7" s="6">
         <f>'Loan Inputs'!B5</f>
@@ -1308,10 +1334,10 @@
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F7" cm="1">
         <f t="array" ref="F7">_xll.QS.TRADE.LOAN("Loans.Case7",Market!$B$3,'Loan Inputs'!$B$7,'Loan Inputs'!$B$8,'Loan Inputs'!$B$11,'Loan Inputs'!$B$4,B7,C7,D7,'Loan Inputs'!$B$9,'Loan Inputs'!$B$10,"Receive",E7)</f>
@@ -1326,26 +1352,26 @@
         <v>0</v>
       </c>
       <c r="I7" s="6" cm="1">
-        <f t="array" ref="I7">_xll.QS.FAIR.RATE(F7,Market!$F$11)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
+        <f t="array" ref="I7">_xll.QS.FAIR.RATE(F7,Market!$F$11,TRUE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B8" s="6">
         <f>'Loan Inputs'!B6</f>
         <v>0</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F8" cm="1">
         <f t="array" ref="F8">_xll.QS.TRADE.LOAN("Loans.Case8",Market!$B$3,'Loan Inputs'!$B$7,'Loan Inputs'!$B$8,'Loan Inputs'!$B$11,'Loan Inputs'!$B$4,B8,C8,D8,'Loan Inputs'!$B$9,'Loan Inputs'!$B$10,"Receive",E8)</f>
@@ -1360,26 +1386,26 @@
         <v>0</v>
       </c>
       <c r="I8" s="6" cm="1">
-        <f t="array" ref="I8">_xll.QS.FAIR.RATE(F8,Market!$F$11)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
+        <f t="array" ref="I8">_xll.QS.FAIR.RATE(F8,Market!$F$11,TRUE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B9" s="6">
         <f>'Loan Inputs'!B6</f>
         <v>0</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F9" cm="1">
         <f t="array" ref="F9">_xll.QS.TRADE.LOAN("Loans.Case9",Market!$B$3,'Loan Inputs'!$B$7,'Loan Inputs'!$B$8,'Loan Inputs'!$B$11,'Loan Inputs'!$B$4,B9,C9,D9,'Loan Inputs'!$B$9,'Loan Inputs'!$B$10,"Receive",E9)</f>
@@ -1393,26 +1419,27 @@
         <f>G9-'Loan Inputs'!$B$4</f>
         <v>0</v>
       </c>
-      <c r="I9" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
+      <c r="I9" s="6" cm="1">
+        <f t="array" ref="I9">_xll.QS.FAIR.RATE(F9,Market!$F$11,TRUE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B10" s="6">
         <f>'Loan Inputs'!B6</f>
         <v>0</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F10" cm="1">
         <f t="array" ref="F10">_xll.QS.TRADE.LOAN("Loans.Case10",Market!$B$3,'Loan Inputs'!$B$7,'Loan Inputs'!$B$8,'Loan Inputs'!$B$11,'Loan Inputs'!$B$4,B10,C10,D10,'Loan Inputs'!$B$9,'Loan Inputs'!$B$10,"Receive",E10)</f>
@@ -1426,13 +1453,13 @@
         <f>G10-'Loan Inputs'!$B$4</f>
         <v>0</v>
       </c>
-      <c r="I10" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9">
+      <c r="I10" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B11" s="6">
         <f>'Loan Inputs'!B5</f>
@@ -1440,10 +1467,10 @@
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F11" cm="1">
         <f t="array" ref="F11">_xll.QS.TRADE.LOAN("Loans.Case11",Market!$B$3,'Loan Inputs'!$B$7,'Loan Inputs'!$B$8,'Loan Inputs'!$B$11,'Loan Inputs'!$B$4,B11,C11,D11,'Loan Inputs'!$B$9,'Loan Inputs'!$B$10,"Receive",E11)</f>
@@ -1458,13 +1485,13 @@
         <v>0</v>
       </c>
       <c r="I11" s="6" cm="1">
-        <f t="array" ref="I11">_xll.QS.FAIR.RATE(F11,Market!$F$11)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
+        <f t="array" ref="I11">_xll.QS.FAIR.RATE(F11,Market!$F$11,TRUE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B12" s="6">
         <f>'Loan Inputs'!B5</f>
@@ -1472,10 +1499,10 @@
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F12" cm="1">
         <f t="array" ref="F12">_xll.QS.TRADE.LOAN("Loans.Case12",Market!$B$3,'Loan Inputs'!$B$7,'Loan Inputs'!$B$8,'Loan Inputs'!$B$11,'Loan Inputs'!$B$4,B12,C12,D12,'Loan Inputs'!$B$9,'Loan Inputs'!$B$10,"Receive",E12)</f>
@@ -1490,13 +1517,13 @@
         <v>0</v>
       </c>
       <c r="I12" s="6" cm="1">
-        <f t="array" ref="I12">_xll.QS.FAIR.RATE(F12,Market!$F$11)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
+        <f t="array" ref="I12">_xll.QS.FAIR.RATE(F12,Market!$F$11,TRUE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B13" s="6">
         <f>'Loan Inputs'!B5</f>
@@ -1504,10 +1531,10 @@
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F13" cm="1">
         <f t="array" ref="F13">_xll.QS.TRADE.LOAN("Loans.Case13",Market!$B$3,'Loan Inputs'!$B$7,'Loan Inputs'!$B$8,'Loan Inputs'!$B$11,'Loan Inputs'!$B$4,B13,C13,D13,'Loan Inputs'!$B$9,'Loan Inputs'!$B$10,"Receive",E13)</f>
@@ -1522,26 +1549,26 @@
         <v>0</v>
       </c>
       <c r="I13" s="6" cm="1">
-        <f t="array" ref="I13">_xll.QS.FAIR.RATE(F13,Market!$F$11)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
+        <f t="array" ref="I13">_xll.QS.FAIR.RATE(F13,Market!$F$11,TRUE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B14" s="6">
         <f>'Loan Inputs'!B6</f>
         <v>0</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F14" cm="1">
         <f t="array" ref="F14">_xll.QS.TRADE.LOAN("Loans.Case14",Market!$B$3,'Loan Inputs'!$B$7,'Loan Inputs'!$B$8,'Loan Inputs'!$B$11,'Loan Inputs'!$B$4,B14,C14,D14,'Loan Inputs'!$B$9,'Loan Inputs'!$B$10,"Receive",E14)</f>
@@ -1556,7 +1583,69 @@
         <v>0</v>
       </c>
       <c r="I14" s="6" cm="1">
-        <f t="array" ref="I14">_xll.QS.FAIR.RATE(F14,Market!$F$11)</f>
+        <f t="array" ref="I14">_xll.QS.FAIR.RATE(F14,Market!$F$11,TRUE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" s="6">
+        <v>0.03</v>
+      </c>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F15" cm="1">
+        <f t="array" ref="F15">_xll.QS.TRADE.LOAN("Loans.Case15",Market!$B$3,'Loan Inputs'!$B$7,'Loan Inputs'!$B$8,'Loan Inputs'!$B$11,'Loan Inputs'!$B$4,B15,C15,D15,'Loan Inputs'!$B$9,'Loan Inputs'!$B$10,"Receive",E15)</f>
+        <v>0</v>
+      </c>
+      <c r="G15" s="7" cm="1">
+        <f t="array" ref="G15">_xll.QS.PRICE(F15,Market!$F$11)</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="7">
+        <f>G15-'Loan Inputs'!$B$4</f>
+        <v>0</v>
+      </c>
+      <c r="I15" s="6" cm="1">
+        <f t="array" ref="I15">_xll.QS.FAIR.RATE(F15,Market!$F$11,TRUE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" t="s">
+        <v>93</v>
+      </c>
+      <c r="B16" s="6">
+        <v>0.03</v>
+      </c>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F16" cm="1">
+        <f t="array" ref="F16">_xll.QS.TRADE.LOAN("Loans.Case16",Market!$B$3,'Loan Inputs'!$B$7,'Loan Inputs'!$B$8,'Loan Inputs'!$B$11,'Loan Inputs'!$B$4,B16,C16,D16,'Loan Inputs'!$B$9,'Loan Inputs'!$B$10,"Receive",E16)</f>
+        <v>0</v>
+      </c>
+      <c r="G16" s="7" cm="1">
+        <f t="array" ref="G16">_xll.QS.PRICE(F16,Market!$F$11)</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="7">
+        <f>G16-'Loan Inputs'!$B$4</f>
+        <v>0</v>
+      </c>
+      <c r="I16" s="6" cm="1">
+        <f t="array" ref="I16">_xll.QS.FAIR.RATE(F16,Market!$F$11,TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -1575,10 +1664,10 @@
   <sheetData>
     <row r="2" spans="1:11">
       <c r="A2" s="8" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -1606,10 +1695,10 @@
   <sheetData>
     <row r="2" spans="1:5">
       <c r="A2" s="8" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1624,7 +1713,7 @@
     </row>
     <row r="25" spans="1:1">
       <c r="A25" s="1" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1642,7 +1731,7 @@
   <sheetData>
     <row r="2" spans="1:1">
       <c r="A2" s="8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:1">
@@ -1653,7 +1742,7 @@
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="8" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="1:1">
@@ -1664,7 +1753,7 @@
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="8" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
     </row>
     <row r="18" spans="1:1">

</xml_diff>